<commit_message>
#26 eSpark BOM added
</commit_message>
<xml_diff>
--- a/Design Files/Relay-Driver-Board-v1.0/BOM/eSpark-BOM-Relay-Driver-Board-v1.0.xlsx
+++ b/Design Files/Relay-Driver-Board-v1.0/BOM/eSpark-BOM-Relay-Driver-Board-v1.0.xlsx
@@ -2265,17 +2265,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2302,6 +2291,17 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2624,14 +2624,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2823,7 +2823,7 @@
       <c r="J8" s="14" t="s">
         <v>415</v>
       </c>
-      <c r="K8" s="45" t="s">
+      <c r="K8" s="42" t="s">
         <v>505</v>
       </c>
       <c r="L8" s="14">
@@ -2836,7 +2836,7 @@
       <c r="N8" s="20">
         <v>80</v>
       </c>
-      <c r="O8" s="52" t="s">
+      <c r="O8" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P8" s="21">
@@ -2866,7 +2866,7 @@
       <c r="F9" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="46" t="s">
         <v>286</v>
       </c>
       <c r="H9" s="20" t="s">
@@ -2878,7 +2878,7 @@
       <c r="J9" s="20" t="s">
         <v>590</v>
       </c>
-      <c r="K9" s="46" t="s">
+      <c r="K9" s="43" t="s">
         <v>506</v>
       </c>
       <c r="L9" s="20">
@@ -2891,7 +2891,7 @@
       <c r="N9" s="20">
         <v>50</v>
       </c>
-      <c r="O9" s="52" t="s">
+      <c r="O9" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P9" s="21">
@@ -2933,7 +2933,7 @@
       <c r="J10" s="14" t="s">
         <v>416</v>
       </c>
-      <c r="K10" s="45" t="s">
+      <c r="K10" s="42" t="s">
         <v>507</v>
       </c>
       <c r="L10" s="14">
@@ -2946,7 +2946,7 @@
       <c r="N10" s="14">
         <v>6</v>
       </c>
-      <c r="O10" s="53" t="s">
+      <c r="O10" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P10" s="15">
@@ -2976,7 +2976,7 @@
       <c r="F11" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="G11" s="49" t="s">
+      <c r="G11" s="46" t="s">
         <v>287</v>
       </c>
       <c r="H11" s="20" t="s">
@@ -2988,7 +2988,7 @@
       <c r="J11" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="K11" s="46" t="s">
+      <c r="K11" s="43" t="s">
         <v>508</v>
       </c>
       <c r="L11" s="20">
@@ -3001,7 +3001,7 @@
       <c r="N11" s="20">
         <v>100</v>
       </c>
-      <c r="O11" s="53" t="s">
+      <c r="O11" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P11" s="21">
@@ -3043,7 +3043,7 @@
       <c r="J12" s="14" t="s">
         <v>417</v>
       </c>
-      <c r="K12" s="45" t="s">
+      <c r="K12" s="42" t="s">
         <v>509</v>
       </c>
       <c r="L12" s="14">
@@ -3056,7 +3056,7 @@
       <c r="N12" s="14">
         <v>50</v>
       </c>
-      <c r="O12" s="53" t="s">
+      <c r="O12" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P12" s="15">
@@ -3098,7 +3098,7 @@
       <c r="J13" s="20" t="s">
         <v>418</v>
       </c>
-      <c r="K13" s="46" t="s">
+      <c r="K13" s="43" t="s">
         <v>510</v>
       </c>
       <c r="L13" s="20">
@@ -3111,7 +3111,7 @@
       <c r="N13" s="20">
         <v>100</v>
       </c>
-      <c r="O13" s="53" t="s">
+      <c r="O13" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P13" s="21">
@@ -3153,7 +3153,7 @@
       <c r="J14" s="14" t="s">
         <v>419</v>
       </c>
-      <c r="K14" s="45" t="s">
+      <c r="K14" s="42" t="s">
         <v>507</v>
       </c>
       <c r="L14" s="14">
@@ -3164,9 +3164,9 @@
         <v>15</v>
       </c>
       <c r="N14" s="14">
-        <v>11</v>
-      </c>
-      <c r="O14" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="O14" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P14" s="15">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="Q14" s="15">
         <f>P14*N14</f>
-        <v>11.325600000000001</v>
+        <v>16.473600000000001</v>
       </c>
       <c r="R14" s="14"/>
     </row>
@@ -3208,7 +3208,7 @@
       <c r="J15" s="20" t="s">
         <v>420</v>
       </c>
-      <c r="K15" s="46" t="s">
+      <c r="K15" s="43" t="s">
         <v>511</v>
       </c>
       <c r="L15" s="20">
@@ -3221,7 +3221,7 @@
       <c r="N15" s="14">
         <v>100</v>
       </c>
-      <c r="O15" s="53" t="s">
+      <c r="O15" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P15" s="15">
@@ -3263,7 +3263,7 @@
       <c r="J16" s="14" t="s">
         <v>421</v>
       </c>
-      <c r="K16" s="45" t="s">
+      <c r="K16" s="42" t="s">
         <v>512</v>
       </c>
       <c r="L16" s="14">
@@ -3276,7 +3276,7 @@
       <c r="N16" s="14">
         <v>6</v>
       </c>
-      <c r="O16" s="53" t="s">
+      <c r="O16" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P16" s="15">
@@ -3318,7 +3318,7 @@
       <c r="J17" s="20" t="s">
         <v>422</v>
       </c>
-      <c r="K17" s="46" t="s">
+      <c r="K17" s="43" t="s">
         <v>513</v>
       </c>
       <c r="L17" s="20">
@@ -3331,7 +3331,7 @@
       <c r="N17" s="20">
         <v>100</v>
       </c>
-      <c r="O17" s="53" t="s">
+      <c r="O17" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P17" s="21">
@@ -3373,7 +3373,7 @@
       <c r="J18" s="14" t="s">
         <v>423</v>
       </c>
-      <c r="K18" s="45" t="s">
+      <c r="K18" s="42" t="s">
         <v>514</v>
       </c>
       <c r="L18" s="14">
@@ -3386,7 +3386,7 @@
       <c r="N18" s="20">
         <v>10</v>
       </c>
-      <c r="O18" s="53" t="s">
+      <c r="O18" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P18" s="21">
@@ -3428,7 +3428,7 @@
       <c r="J19" s="20" t="s">
         <v>584</v>
       </c>
-      <c r="K19" s="46" t="s">
+      <c r="K19" s="43" t="s">
         <v>515</v>
       </c>
       <c r="L19" s="20">
@@ -3441,7 +3441,7 @@
       <c r="N19" s="20">
         <v>100</v>
       </c>
-      <c r="O19" s="53" t="s">
+      <c r="O19" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P19" s="21">
@@ -3483,7 +3483,7 @@
       <c r="J20" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="K20" s="45" t="s">
+      <c r="K20" s="42" t="s">
         <v>516</v>
       </c>
       <c r="L20" s="14">
@@ -3496,7 +3496,7 @@
       <c r="N20" s="14">
         <v>50</v>
       </c>
-      <c r="O20" s="53" t="s">
+      <c r="O20" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P20" s="15">
@@ -3517,50 +3517,50 @@
       <c r="C21" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="48" t="s">
+      <c r="D21" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="E21" s="48" t="s">
+      <c r="E21" s="45" t="s">
         <v>145</v>
       </c>
-      <c r="F21" s="48" t="s">
+      <c r="F21" s="45" t="s">
         <v>237</v>
       </c>
-      <c r="G21" s="48" t="s">
+      <c r="G21" s="45" t="s">
         <v>295</v>
       </c>
-      <c r="H21" s="48" t="s">
+      <c r="H21" s="45" t="s">
         <v>374</v>
       </c>
       <c r="I21" s="14" t="s">
         <v>439</v>
       </c>
-      <c r="J21" s="48" t="s">
+      <c r="J21" s="45" t="s">
         <v>425</v>
       </c>
-      <c r="K21" s="47" t="s">
+      <c r="K21" s="44" t="s">
         <v>517</v>
       </c>
-      <c r="L21" s="48">
+      <c r="L21" s="45">
         <v>2</v>
       </c>
-      <c r="M21" s="48">
+      <c r="M21" s="45">
         <f t="shared" ref="M21" si="13">L21*5</f>
         <v>10</v>
       </c>
-      <c r="N21" s="48" t="s">
-        <v>439</v>
-      </c>
-      <c r="O21" s="49" t="s">
-        <v>576</v>
-      </c>
-      <c r="P21" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q21" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="R21" s="51" t="s">
+      <c r="N21" s="45" t="s">
+        <v>439</v>
+      </c>
+      <c r="O21" s="46" t="s">
+        <v>576</v>
+      </c>
+      <c r="P21" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q21" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="R21" s="48" t="s">
         <v>575</v>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
       <c r="J22" s="14" t="s">
         <v>426</v>
       </c>
-      <c r="K22" s="45" t="s">
+      <c r="K22" s="42" t="s">
         <v>518</v>
       </c>
       <c r="L22" s="14">
@@ -3607,7 +3607,7 @@
       <c r="N22" s="20">
         <v>20</v>
       </c>
-      <c r="O22" s="52" t="s">
+      <c r="O22" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P22" s="21">
@@ -3649,7 +3649,7 @@
       <c r="J23" s="20" t="s">
         <v>427</v>
       </c>
-      <c r="K23" s="46" t="s">
+      <c r="K23" s="43" t="s">
         <v>519</v>
       </c>
       <c r="L23" s="20">
@@ -3662,7 +3662,7 @@
       <c r="N23" s="14">
         <v>100</v>
       </c>
-      <c r="O23" s="53" t="s">
+      <c r="O23" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P23" s="15">
@@ -3704,7 +3704,7 @@
       <c r="J24" s="14" t="s">
         <v>428</v>
       </c>
-      <c r="K24" s="45" t="s">
+      <c r="K24" s="42" t="s">
         <v>520</v>
       </c>
       <c r="L24" s="14">
@@ -3717,7 +3717,7 @@
       <c r="N24" s="14">
         <v>50</v>
       </c>
-      <c r="O24" s="52" t="s">
+      <c r="O24" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P24" s="15">
@@ -3759,7 +3759,7 @@
       <c r="J25" s="20" t="s">
         <v>577</v>
       </c>
-      <c r="K25" s="46" t="s">
+      <c r="K25" s="43" t="s">
         <v>518</v>
       </c>
       <c r="L25" s="20">
@@ -3772,7 +3772,7 @@
       <c r="N25" s="20">
         <v>100</v>
       </c>
-      <c r="O25" s="52" t="s">
+      <c r="O25" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P25" s="21">
@@ -3814,7 +3814,7 @@
       <c r="J26" s="14" t="s">
         <v>429</v>
       </c>
-      <c r="K26" s="45" t="s">
+      <c r="K26" s="42" t="s">
         <v>521</v>
       </c>
       <c r="L26" s="14">
@@ -3827,7 +3827,7 @@
       <c r="N26" s="14">
         <v>50</v>
       </c>
-      <c r="O26" s="52" t="s">
+      <c r="O26" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P26" s="15">
@@ -3869,7 +3869,7 @@
       <c r="J27" s="20" t="s">
         <v>430</v>
       </c>
-      <c r="K27" s="46" t="s">
+      <c r="K27" s="43" t="s">
         <v>522</v>
       </c>
       <c r="L27" s="20">
@@ -3882,7 +3882,7 @@
       <c r="N27" s="20">
         <v>100</v>
       </c>
-      <c r="O27" s="52" t="s">
+      <c r="O27" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P27" s="21">
@@ -3924,7 +3924,7 @@
       <c r="J28" s="14" t="s">
         <v>431</v>
       </c>
-      <c r="K28" s="45" t="s">
+      <c r="K28" s="42" t="s">
         <v>523</v>
       </c>
       <c r="L28" s="14">
@@ -3937,7 +3937,7 @@
       <c r="N28" s="14">
         <v>10</v>
       </c>
-      <c r="O28" s="53" t="s">
+      <c r="O28" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P28" s="15">
@@ -3979,7 +3979,7 @@
       <c r="J29" s="20" t="s">
         <v>432</v>
       </c>
-      <c r="K29" s="46" t="s">
+      <c r="K29" s="43" t="s">
         <v>524</v>
       </c>
       <c r="L29" s="20">
@@ -3992,7 +3992,7 @@
       <c r="N29" s="20">
         <v>20</v>
       </c>
-      <c r="O29" s="53" t="s">
+      <c r="O29" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P29" s="21">
@@ -4013,50 +4013,50 @@
       <c r="C30" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="D30" s="48" t="s">
+      <c r="D30" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="48" t="s">
+      <c r="E30" s="45" t="s">
         <v>154</v>
       </c>
-      <c r="F30" s="48" t="s">
+      <c r="F30" s="45" t="s">
         <v>237</v>
       </c>
-      <c r="G30" s="48" t="s">
+      <c r="G30" s="45" t="s">
         <v>304</v>
       </c>
-      <c r="H30" s="48" t="s">
+      <c r="H30" s="45" t="s">
         <v>376</v>
       </c>
       <c r="I30" s="14" t="s">
         <v>439</v>
       </c>
-      <c r="J30" s="48" t="s">
+      <c r="J30" s="45" t="s">
         <v>433</v>
       </c>
-      <c r="K30" s="47" t="s">
+      <c r="K30" s="44" t="s">
         <v>517</v>
       </c>
-      <c r="L30" s="48">
+      <c r="L30" s="45">
         <v>8</v>
       </c>
-      <c r="M30" s="48">
+      <c r="M30" s="45">
         <f>L30*5</f>
         <v>40</v>
       </c>
-      <c r="N30" s="48" t="s">
-        <v>439</v>
-      </c>
-      <c r="O30" s="49" t="s">
-        <v>576</v>
-      </c>
-      <c r="P30" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q30" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="R30" s="51" t="s">
+      <c r="N30" s="45" t="s">
+        <v>439</v>
+      </c>
+      <c r="O30" s="46" t="s">
+        <v>576</v>
+      </c>
+      <c r="P30" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q30" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="R30" s="48" t="s">
         <v>575</v>
       </c>
     </row>
@@ -4090,7 +4090,7 @@
       <c r="J31" s="20" t="s">
         <v>434</v>
       </c>
-      <c r="K31" s="46" t="s">
+      <c r="K31" s="43" t="s">
         <v>525</v>
       </c>
       <c r="L31" s="20">
@@ -4103,7 +4103,7 @@
       <c r="N31" s="14">
         <v>20</v>
       </c>
-      <c r="O31" s="52" t="s">
+      <c r="O31" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P31" s="15">
@@ -4145,7 +4145,7 @@
       <c r="J32" s="14" t="s">
         <v>435</v>
       </c>
-      <c r="K32" s="45" t="s">
+      <c r="K32" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L32" s="14">
@@ -4158,7 +4158,7 @@
       <c r="N32" s="14">
         <v>50</v>
       </c>
-      <c r="O32" s="53" t="s">
+      <c r="O32" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P32" s="15">
@@ -4200,7 +4200,7 @@
       <c r="J33" s="20" t="s">
         <v>585</v>
       </c>
-      <c r="K33" s="45" t="s">
+      <c r="K33" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L33" s="20">
@@ -4213,7 +4213,7 @@
       <c r="N33" s="20">
         <v>15</v>
       </c>
-      <c r="O33" s="53" t="s">
+      <c r="O33" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P33" s="21">
@@ -4255,7 +4255,7 @@
       <c r="J34" s="14" t="s">
         <v>436</v>
       </c>
-      <c r="K34" s="45" t="s">
+      <c r="K34" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L34" s="14">
@@ -4268,7 +4268,7 @@
       <c r="N34" s="14">
         <v>6</v>
       </c>
-      <c r="O34" s="53" t="s">
+      <c r="O34" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P34" s="15">
@@ -4310,7 +4310,7 @@
       <c r="J35" s="20" t="s">
         <v>437</v>
       </c>
-      <c r="K35" s="45" t="s">
+      <c r="K35" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L35" s="20">
@@ -4323,7 +4323,7 @@
       <c r="N35" s="20">
         <v>10</v>
       </c>
-      <c r="O35" s="53" t="s">
+      <c r="O35" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P35" s="21">
@@ -4365,7 +4365,7 @@
       <c r="J36" s="14" t="s">
         <v>438</v>
       </c>
-      <c r="K36" s="45" t="s">
+      <c r="K36" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L36" s="14">
@@ -4378,7 +4378,7 @@
       <c r="N36" s="14">
         <v>15</v>
       </c>
-      <c r="O36" s="53" t="s">
+      <c r="O36" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P36" s="15">
@@ -4420,7 +4420,7 @@
       <c r="J37" s="20" t="s">
         <v>596</v>
       </c>
-      <c r="K37" s="45" t="s">
+      <c r="K37" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L37" s="20">
@@ -4433,7 +4433,7 @@
       <c r="N37" s="20">
         <v>20</v>
       </c>
-      <c r="O37" s="53" t="s">
+      <c r="O37" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P37" s="21">
@@ -4475,7 +4475,7 @@
       <c r="J38" s="14" t="s">
         <v>440</v>
       </c>
-      <c r="K38" s="45" t="s">
+      <c r="K38" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L38" s="14">
@@ -4488,7 +4488,7 @@
       <c r="N38" s="14">
         <v>20</v>
       </c>
-      <c r="O38" s="53" t="s">
+      <c r="O38" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P38" s="15">
@@ -4530,7 +4530,7 @@
       <c r="J39" s="20" t="s">
         <v>441</v>
       </c>
-      <c r="K39" s="45" t="s">
+      <c r="K39" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L39" s="20">
@@ -4543,7 +4543,7 @@
       <c r="N39" s="20">
         <v>20</v>
       </c>
-      <c r="O39" s="53" t="s">
+      <c r="O39" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P39" s="21">
@@ -4585,7 +4585,7 @@
       <c r="J40" s="14" t="s">
         <v>442</v>
       </c>
-      <c r="K40" s="45" t="s">
+      <c r="K40" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L40" s="14">
@@ -4598,7 +4598,7 @@
       <c r="N40" s="14">
         <v>50</v>
       </c>
-      <c r="O40" s="53" t="s">
+      <c r="O40" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P40" s="15">
@@ -4640,7 +4640,7 @@
       <c r="J41" s="20" t="s">
         <v>443</v>
       </c>
-      <c r="K41" s="45" t="s">
+      <c r="K41" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L41" s="20">
@@ -4653,7 +4653,7 @@
       <c r="N41" s="20">
         <v>50</v>
       </c>
-      <c r="O41" s="53" t="s">
+      <c r="O41" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P41" s="21">
@@ -4695,7 +4695,7 @@
       <c r="J42" s="14" t="s">
         <v>444</v>
       </c>
-      <c r="K42" s="45" t="s">
+      <c r="K42" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L42" s="14">
@@ -4708,7 +4708,7 @@
       <c r="N42" s="14">
         <v>15</v>
       </c>
-      <c r="O42" s="53" t="s">
+      <c r="O42" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P42" s="15">
@@ -4750,7 +4750,7 @@
       <c r="J43" s="20" t="s">
         <v>445</v>
       </c>
-      <c r="K43" s="45" t="s">
+      <c r="K43" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L43" s="20">
@@ -4763,7 +4763,7 @@
       <c r="N43" s="20">
         <v>15</v>
       </c>
-      <c r="O43" s="53" t="s">
+      <c r="O43" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P43" s="21">
@@ -4805,7 +4805,7 @@
       <c r="J44" s="14" t="s">
         <v>446</v>
       </c>
-      <c r="K44" s="45" t="s">
+      <c r="K44" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L44" s="14">
@@ -4818,7 +4818,7 @@
       <c r="N44" s="14">
         <v>10</v>
       </c>
-      <c r="O44" s="53" t="s">
+      <c r="O44" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P44" s="15">
@@ -4860,7 +4860,7 @@
       <c r="J45" s="20" t="s">
         <v>447</v>
       </c>
-      <c r="K45" s="45" t="s">
+      <c r="K45" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L45" s="20">
@@ -4873,7 +4873,7 @@
       <c r="N45" s="14">
         <v>20</v>
       </c>
-      <c r="O45" s="53" t="s">
+      <c r="O45" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P45" s="15">
@@ -4903,7 +4903,7 @@
       <c r="F46" s="14" t="s">
         <v>253</v>
       </c>
-      <c r="G46" s="48" t="s">
+      <c r="G46" s="45" t="s">
         <v>526</v>
       </c>
       <c r="H46" s="14" t="s">
@@ -4915,7 +4915,7 @@
       <c r="J46" s="14" t="s">
         <v>580</v>
       </c>
-      <c r="K46" s="45" t="s">
+      <c r="K46" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L46" s="14">
@@ -4928,7 +4928,7 @@
       <c r="N46" s="14">
         <v>50</v>
       </c>
-      <c r="O46" s="52" t="s">
+      <c r="O46" s="49" t="s">
         <v>576</v>
       </c>
       <c r="P46" s="15">
@@ -4970,7 +4970,7 @@
       <c r="J47" s="20" t="s">
         <v>448</v>
       </c>
-      <c r="K47" s="45" t="s">
+      <c r="K47" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L47" s="20">
@@ -4983,7 +4983,7 @@
       <c r="N47" s="14">
         <v>10</v>
       </c>
-      <c r="O47" s="53" t="s">
+      <c r="O47" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P47" s="15">
@@ -5025,7 +5025,7 @@
       <c r="J48" s="14" t="s">
         <v>449</v>
       </c>
-      <c r="K48" s="45" t="s">
+      <c r="K48" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L48" s="14">
@@ -5038,7 +5038,7 @@
       <c r="N48" s="14">
         <v>11</v>
       </c>
-      <c r="O48" s="53" t="s">
+      <c r="O48" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P48" s="15">
@@ -5080,7 +5080,7 @@
       <c r="J49" s="20" t="s">
         <v>586</v>
       </c>
-      <c r="K49" s="45" t="s">
+      <c r="K49" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L49" s="20">
@@ -5093,7 +5093,7 @@
       <c r="N49" s="20">
         <v>100</v>
       </c>
-      <c r="O49" s="53" t="s">
+      <c r="O49" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P49" s="21">
@@ -5135,7 +5135,7 @@
       <c r="J50" s="14" t="s">
         <v>450</v>
       </c>
-      <c r="K50" s="45" t="s">
+      <c r="K50" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L50" s="14">
@@ -5148,7 +5148,7 @@
       <c r="N50" s="14">
         <v>10</v>
       </c>
-      <c r="O50" s="53" t="s">
+      <c r="O50" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P50" s="15">
@@ -5190,7 +5190,7 @@
       <c r="J51" s="14" t="s">
         <v>581</v>
       </c>
-      <c r="K51" s="45" t="s">
+      <c r="K51" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L51" s="20">
@@ -5203,7 +5203,7 @@
       <c r="N51" s="14">
         <v>16</v>
       </c>
-      <c r="O51" s="53" t="s">
+      <c r="O51" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P51" s="15">
@@ -5245,7 +5245,7 @@
       <c r="J52" s="14" t="s">
         <v>451</v>
       </c>
-      <c r="K52" s="45" t="s">
+      <c r="K52" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L52" s="14">
@@ -5258,7 +5258,7 @@
       <c r="N52" s="14">
         <v>21</v>
       </c>
-      <c r="O52" s="53" t="s">
+      <c r="O52" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P52" s="15">
@@ -5298,7 +5298,7 @@
       <c r="J53" s="20" t="s">
         <v>582</v>
       </c>
-      <c r="K53" s="45" t="s">
+      <c r="K53" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L53" s="20">
@@ -5311,7 +5311,7 @@
       <c r="N53" s="20">
         <v>10</v>
       </c>
-      <c r="O53" s="53" t="s">
+      <c r="O53" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P53" s="21">
@@ -5353,7 +5353,7 @@
       <c r="J54" s="14" t="s">
         <v>452</v>
       </c>
-      <c r="K54" s="45" t="s">
+      <c r="K54" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L54" s="14">
@@ -5366,7 +5366,7 @@
       <c r="N54" s="14">
         <v>85</v>
       </c>
-      <c r="O54" s="53" t="s">
+      <c r="O54" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P54" s="15">
@@ -5408,7 +5408,7 @@
       <c r="J55" s="20" t="s">
         <v>453</v>
       </c>
-      <c r="K55" s="46" t="s">
+      <c r="K55" s="43" t="s">
         <v>527</v>
       </c>
       <c r="L55" s="20">
@@ -5421,7 +5421,7 @@
       <c r="N55" s="20">
         <v>6</v>
       </c>
-      <c r="O55" s="53" t="s">
+      <c r="O55" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P55" s="21">
@@ -5463,7 +5463,7 @@
       <c r="J56" s="14" t="s">
         <v>454</v>
       </c>
-      <c r="K56" s="45" t="s">
+      <c r="K56" s="42" t="s">
         <v>528</v>
       </c>
       <c r="L56" s="14">
@@ -5476,7 +5476,7 @@
       <c r="N56" s="14">
         <v>6</v>
       </c>
-      <c r="O56" s="53" t="s">
+      <c r="O56" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P56" s="15">
@@ -5518,7 +5518,7 @@
       <c r="J57" s="20" t="s">
         <v>455</v>
       </c>
-      <c r="K57" s="46" t="s">
+      <c r="K57" s="43" t="s">
         <v>529</v>
       </c>
       <c r="L57" s="20">
@@ -5531,7 +5531,7 @@
       <c r="N57" s="20">
         <v>10</v>
       </c>
-      <c r="O57" s="53" t="s">
+      <c r="O57" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P57" s="21">
@@ -5573,7 +5573,7 @@
       <c r="J58" s="14" t="s">
         <v>456</v>
       </c>
-      <c r="K58" s="45" t="s">
+      <c r="K58" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L58" s="14">
@@ -5586,7 +5586,7 @@
       <c r="N58" s="20">
         <v>100</v>
       </c>
-      <c r="O58" s="53" t="s">
+      <c r="O58" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P58" s="21">
@@ -5628,7 +5628,7 @@
       <c r="J59" s="20" t="s">
         <v>457</v>
       </c>
-      <c r="K59" s="45" t="s">
+      <c r="K59" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L59" s="20">
@@ -5641,7 +5641,7 @@
       <c r="N59" s="14">
         <v>40</v>
       </c>
-      <c r="O59" s="53" t="s">
+      <c r="O59" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P59" s="15">
@@ -5683,7 +5683,7 @@
       <c r="J60" s="14" t="s">
         <v>458</v>
       </c>
-      <c r="K60" s="45" t="s">
+      <c r="K60" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L60" s="14">
@@ -5696,7 +5696,7 @@
       <c r="N60" s="20">
         <v>20</v>
       </c>
-      <c r="O60" s="53" t="s">
+      <c r="O60" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P60" s="21">
@@ -5738,7 +5738,7 @@
       <c r="J61" s="20" t="s">
         <v>459</v>
       </c>
-      <c r="K61" s="45" t="s">
+      <c r="K61" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L61" s="20">
@@ -5751,7 +5751,7 @@
       <c r="N61" s="20">
         <v>100</v>
       </c>
-      <c r="O61" s="53" t="s">
+      <c r="O61" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P61" s="21">
@@ -5793,7 +5793,7 @@
       <c r="J62" s="14" t="s">
         <v>460</v>
       </c>
-      <c r="K62" s="45" t="s">
+      <c r="K62" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L62" s="14">
@@ -5806,7 +5806,7 @@
       <c r="N62" s="14">
         <v>11</v>
       </c>
-      <c r="O62" s="53" t="s">
+      <c r="O62" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P62" s="15">
@@ -5848,7 +5848,7 @@
       <c r="J63" s="20" t="s">
         <v>461</v>
       </c>
-      <c r="K63" s="45" t="s">
+      <c r="K63" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L63" s="20">
@@ -5861,7 +5861,7 @@
       <c r="N63" s="20">
         <v>10</v>
       </c>
-      <c r="O63" s="53" t="s">
+      <c r="O63" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P63" s="21">
@@ -5903,7 +5903,7 @@
       <c r="J64" s="14" t="s">
         <v>462</v>
       </c>
-      <c r="K64" s="45" t="s">
+      <c r="K64" s="42" t="s">
         <v>530</v>
       </c>
       <c r="L64" s="14">
@@ -5916,7 +5916,7 @@
       <c r="N64" s="20">
         <v>50</v>
       </c>
-      <c r="O64" s="53" t="s">
+      <c r="O64" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P64" s="21">
@@ -5958,7 +5958,7 @@
       <c r="J65" s="20" t="s">
         <v>463</v>
       </c>
-      <c r="K65" s="46" t="s">
+      <c r="K65" s="43" t="s">
         <v>531</v>
       </c>
       <c r="L65" s="20">
@@ -5971,7 +5971,7 @@
       <c r="N65" s="20">
         <v>6</v>
       </c>
-      <c r="O65" s="53" t="s">
+      <c r="O65" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P65" s="21">
@@ -6013,7 +6013,7 @@
       <c r="J66" s="14" t="s">
         <v>464</v>
       </c>
-      <c r="K66" s="45" t="s">
+      <c r="K66" s="42" t="s">
         <v>532</v>
       </c>
       <c r="L66" s="14">
@@ -6026,7 +6026,7 @@
       <c r="N66" s="14">
         <v>100</v>
       </c>
-      <c r="O66" s="53" t="s">
+      <c r="O66" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P66" s="15">
@@ -6068,7 +6068,7 @@
       <c r="J67" s="20" t="s">
         <v>465</v>
       </c>
-      <c r="K67" s="46" t="s">
+      <c r="K67" s="43" t="s">
         <v>533</v>
       </c>
       <c r="L67" s="20">
@@ -6081,7 +6081,7 @@
       <c r="N67" s="20">
         <v>20</v>
       </c>
-      <c r="O67" s="53" t="s">
+      <c r="O67" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P67" s="21">
@@ -6123,7 +6123,7 @@
       <c r="J68" s="14" t="s">
         <v>466</v>
       </c>
-      <c r="K68" s="45" t="s">
+      <c r="K68" s="42" t="s">
         <v>534</v>
       </c>
       <c r="L68" s="14">
@@ -6136,7 +6136,7 @@
       <c r="N68" s="14">
         <v>100</v>
       </c>
-      <c r="O68" s="53" t="s">
+      <c r="O68" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P68" s="15">
@@ -6178,7 +6178,7 @@
       <c r="J69" s="20" t="s">
         <v>467</v>
       </c>
-      <c r="K69" s="46" t="s">
+      <c r="K69" s="43" t="s">
         <v>535</v>
       </c>
       <c r="L69" s="20">
@@ -6191,7 +6191,7 @@
       <c r="N69" s="20">
         <v>100</v>
       </c>
-      <c r="O69" s="53" t="s">
+      <c r="O69" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P69" s="21">
@@ -6233,7 +6233,7 @@
       <c r="J70" s="14" t="s">
         <v>468</v>
       </c>
-      <c r="K70" s="45" t="s">
+      <c r="K70" s="42" t="s">
         <v>536</v>
       </c>
       <c r="L70" s="14">
@@ -6246,7 +6246,7 @@
       <c r="N70" s="14">
         <v>100</v>
       </c>
-      <c r="O70" s="53" t="s">
+      <c r="O70" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P70" s="15">
@@ -6288,7 +6288,7 @@
       <c r="J71" s="20" t="s">
         <v>469</v>
       </c>
-      <c r="K71" s="46" t="s">
+      <c r="K71" s="43" t="s">
         <v>537</v>
       </c>
       <c r="L71" s="20">
@@ -6301,7 +6301,7 @@
       <c r="N71" s="20">
         <v>100</v>
       </c>
-      <c r="O71" s="53" t="s">
+      <c r="O71" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P71" s="21">
@@ -6343,7 +6343,7 @@
       <c r="J72" s="14" t="s">
         <v>470</v>
       </c>
-      <c r="K72" s="45" t="s">
+      <c r="K72" s="42" t="s">
         <v>538</v>
       </c>
       <c r="L72" s="14">
@@ -6356,7 +6356,7 @@
       <c r="N72" s="14">
         <v>100</v>
       </c>
-      <c r="O72" s="53" t="s">
+      <c r="O72" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P72" s="15">
@@ -6398,7 +6398,7 @@
       <c r="J73" s="20" t="s">
         <v>471</v>
       </c>
-      <c r="K73" s="46" t="s">
+      <c r="K73" s="43" t="s">
         <v>539</v>
       </c>
       <c r="L73" s="20">
@@ -6411,7 +6411,7 @@
       <c r="N73" s="20">
         <v>100</v>
       </c>
-      <c r="O73" s="53" t="s">
+      <c r="O73" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P73" s="21">
@@ -6453,7 +6453,7 @@
       <c r="J74" s="14" t="s">
         <v>472</v>
       </c>
-      <c r="K74" s="45" t="s">
+      <c r="K74" s="42" t="s">
         <v>540</v>
       </c>
       <c r="L74" s="14">
@@ -6466,7 +6466,7 @@
       <c r="N74" s="14">
         <v>100</v>
       </c>
-      <c r="O74" s="53" t="s">
+      <c r="O74" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P74" s="15">
@@ -6508,7 +6508,7 @@
       <c r="J75" s="20" t="s">
         <v>473</v>
       </c>
-      <c r="K75" s="46" t="s">
+      <c r="K75" s="43" t="s">
         <v>541</v>
       </c>
       <c r="L75" s="20">
@@ -6521,7 +6521,7 @@
       <c r="N75" s="20">
         <v>100</v>
       </c>
-      <c r="O75" s="53" t="s">
+      <c r="O75" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P75" s="21">
@@ -6563,7 +6563,7 @@
       <c r="J76" s="14" t="s">
         <v>474</v>
       </c>
-      <c r="K76" s="45" t="s">
+      <c r="K76" s="42" t="s">
         <v>542</v>
       </c>
       <c r="L76" s="14">
@@ -6576,7 +6576,7 @@
       <c r="N76" s="14">
         <v>100</v>
       </c>
-      <c r="O76" s="53" t="s">
+      <c r="O76" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P76" s="15">
@@ -6618,7 +6618,7 @@
       <c r="J77" s="20" t="s">
         <v>475</v>
       </c>
-      <c r="K77" s="46" t="s">
+      <c r="K77" s="43" t="s">
         <v>543</v>
       </c>
       <c r="L77" s="20">
@@ -6631,7 +6631,7 @@
       <c r="N77" s="20">
         <v>20</v>
       </c>
-      <c r="O77" s="53" t="s">
+      <c r="O77" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P77" s="21">
@@ -6673,7 +6673,7 @@
       <c r="J78" s="14" t="s">
         <v>476</v>
       </c>
-      <c r="K78" s="45" t="s">
+      <c r="K78" s="42" t="s">
         <v>544</v>
       </c>
       <c r="L78" s="14">
@@ -6686,7 +6686,7 @@
       <c r="N78" s="14">
         <v>100</v>
       </c>
-      <c r="O78" s="53" t="s">
+      <c r="O78" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P78" s="15">
@@ -6728,7 +6728,7 @@
       <c r="J79" s="20" t="s">
         <v>587</v>
       </c>
-      <c r="K79" s="46" t="s">
+      <c r="K79" s="43" t="s">
         <v>545</v>
       </c>
       <c r="L79" s="20">
@@ -6741,7 +6741,7 @@
       <c r="N79" s="20">
         <v>100</v>
       </c>
-      <c r="O79" s="53" t="s">
+      <c r="O79" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P79" s="21">
@@ -6783,7 +6783,7 @@
       <c r="J80" s="14" t="s">
         <v>477</v>
       </c>
-      <c r="K80" s="45" t="s">
+      <c r="K80" s="42" t="s">
         <v>546</v>
       </c>
       <c r="L80" s="14">
@@ -6796,7 +6796,7 @@
       <c r="N80" s="14">
         <v>100</v>
       </c>
-      <c r="O80" s="53" t="s">
+      <c r="O80" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P80" s="15">
@@ -6838,7 +6838,7 @@
       <c r="J81" s="20" t="s">
         <v>478</v>
       </c>
-      <c r="K81" s="46" t="s">
+      <c r="K81" s="43" t="s">
         <v>547</v>
       </c>
       <c r="L81" s="20">
@@ -6851,7 +6851,7 @@
       <c r="N81" s="20">
         <v>100</v>
       </c>
-      <c r="O81" s="53" t="s">
+      <c r="O81" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P81" s="21">
@@ -6872,50 +6872,50 @@
       <c r="C82" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="D82" s="48" t="s">
+      <c r="D82" s="45" t="s">
         <v>101</v>
       </c>
-      <c r="E82" s="48" t="s">
+      <c r="E82" s="45" t="s">
         <v>205</v>
       </c>
-      <c r="F82" s="48" t="s">
+      <c r="F82" s="45" t="s">
         <v>270</v>
       </c>
-      <c r="G82" s="48" t="s">
+      <c r="G82" s="45" t="s">
         <v>343</v>
       </c>
-      <c r="H82" s="48" t="s">
+      <c r="H82" s="45" t="s">
         <v>374</v>
       </c>
       <c r="I82" s="20" t="s">
         <v>439</v>
       </c>
-      <c r="J82" s="48" t="s">
+      <c r="J82" s="45" t="s">
         <v>479</v>
       </c>
-      <c r="K82" s="47" t="s">
+      <c r="K82" s="44" t="s">
         <v>517</v>
       </c>
-      <c r="L82" s="48">
+      <c r="L82" s="45">
         <v>2</v>
       </c>
-      <c r="M82" s="48">
+      <c r="M82" s="45">
         <f>L82*5</f>
         <v>10</v>
       </c>
-      <c r="N82" s="48" t="s">
-        <v>439</v>
-      </c>
-      <c r="O82" s="49" t="s">
-        <v>576</v>
-      </c>
-      <c r="P82" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q82" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="R82" s="51" t="s">
+      <c r="N82" s="45" t="s">
+        <v>439</v>
+      </c>
+      <c r="O82" s="46" t="s">
+        <v>576</v>
+      </c>
+      <c r="P82" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q82" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="R82" s="48" t="s">
         <v>575</v>
       </c>
     </row>
@@ -6949,7 +6949,7 @@
       <c r="J83" s="20" t="s">
         <v>480</v>
       </c>
-      <c r="K83" s="46" t="s">
+      <c r="K83" s="43" t="s">
         <v>548</v>
       </c>
       <c r="L83" s="20">
@@ -6962,7 +6962,7 @@
       <c r="N83" s="20">
         <v>100</v>
       </c>
-      <c r="O83" s="53" t="s">
+      <c r="O83" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P83" s="21">
@@ -7004,7 +7004,7 @@
       <c r="J84" s="14" t="s">
         <v>481</v>
       </c>
-      <c r="K84" s="45" t="s">
+      <c r="K84" s="42" t="s">
         <v>549</v>
       </c>
       <c r="L84" s="14">
@@ -7017,7 +7017,7 @@
       <c r="N84" s="14">
         <v>100</v>
       </c>
-      <c r="O84" s="53" t="s">
+      <c r="O84" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P84" s="15">
@@ -7059,7 +7059,7 @@
       <c r="J85" s="20" t="s">
         <v>479</v>
       </c>
-      <c r="K85" s="46" t="s">
+      <c r="K85" s="43" t="s">
         <v>532</v>
       </c>
       <c r="L85" s="20">
@@ -7072,7 +7072,7 @@
       <c r="N85" s="20">
         <v>100</v>
       </c>
-      <c r="O85" s="53" t="s">
+      <c r="O85" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P85" s="21">
@@ -7114,7 +7114,7 @@
       <c r="J86" s="14" t="s">
         <v>482</v>
       </c>
-      <c r="K86" s="45" t="s">
+      <c r="K86" s="42" t="s">
         <v>550</v>
       </c>
       <c r="L86" s="14">
@@ -7127,7 +7127,7 @@
       <c r="N86" s="14">
         <v>100</v>
       </c>
-      <c r="O86" s="53" t="s">
+      <c r="O86" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P86" s="15">
@@ -7169,7 +7169,7 @@
       <c r="J87" s="20" t="s">
         <v>483</v>
       </c>
-      <c r="K87" s="46" t="s">
+      <c r="K87" s="43" t="s">
         <v>551</v>
       </c>
       <c r="L87" s="20">
@@ -7182,7 +7182,7 @@
       <c r="N87" s="20">
         <v>100</v>
       </c>
-      <c r="O87" s="53" t="s">
+      <c r="O87" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P87" s="21">
@@ -7224,7 +7224,7 @@
       <c r="J88" s="14" t="s">
         <v>484</v>
       </c>
-      <c r="K88" s="45" t="s">
+      <c r="K88" s="42" t="s">
         <v>552</v>
       </c>
       <c r="L88" s="14">
@@ -7237,7 +7237,7 @@
       <c r="N88" s="14">
         <v>100</v>
       </c>
-      <c r="O88" s="53" t="s">
+      <c r="O88" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P88" s="15">
@@ -7279,7 +7279,7 @@
       <c r="J89" s="20" t="s">
         <v>485</v>
       </c>
-      <c r="K89" s="46" t="s">
+      <c r="K89" s="43" t="s">
         <v>553</v>
       </c>
       <c r="L89" s="20">
@@ -7292,7 +7292,7 @@
       <c r="N89" s="20">
         <v>100</v>
       </c>
-      <c r="O89" s="53" t="s">
+      <c r="O89" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P89" s="21">
@@ -7334,7 +7334,7 @@
       <c r="J90" s="14" t="s">
         <v>486</v>
       </c>
-      <c r="K90" s="45" t="s">
+      <c r="K90" s="42" t="s">
         <v>554</v>
       </c>
       <c r="L90" s="14">
@@ -7347,7 +7347,7 @@
       <c r="N90" s="14">
         <v>100</v>
       </c>
-      <c r="O90" s="53" t="s">
+      <c r="O90" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P90" s="15">
@@ -7389,7 +7389,7 @@
       <c r="J91" s="20" t="s">
         <v>487</v>
       </c>
-      <c r="K91" s="46" t="s">
+      <c r="K91" s="43" t="s">
         <v>555</v>
       </c>
       <c r="L91" s="20">
@@ -7402,7 +7402,7 @@
       <c r="N91" s="20">
         <v>100</v>
       </c>
-      <c r="O91" s="53" t="s">
+      <c r="O91" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P91" s="21">
@@ -7444,7 +7444,7 @@
       <c r="J92" s="14" t="s">
         <v>488</v>
       </c>
-      <c r="K92" s="45" t="s">
+      <c r="K92" s="42" t="s">
         <v>556</v>
       </c>
       <c r="L92" s="14">
@@ -7457,7 +7457,7 @@
       <c r="N92" s="14">
         <v>100</v>
       </c>
-      <c r="O92" s="53" t="s">
+      <c r="O92" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P92" s="15">
@@ -7499,7 +7499,7 @@
       <c r="J93" s="20" t="s">
         <v>489</v>
       </c>
-      <c r="K93" s="46" t="s">
+      <c r="K93" s="43" t="s">
         <v>557</v>
       </c>
       <c r="L93" s="20">
@@ -7512,7 +7512,7 @@
       <c r="N93" s="20">
         <v>50</v>
       </c>
-      <c r="O93" s="53" t="s">
+      <c r="O93" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P93" s="21">
@@ -7533,50 +7533,50 @@
       <c r="C94" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="D94" s="48" t="s">
+      <c r="D94" s="45" t="s">
         <v>113</v>
       </c>
-      <c r="E94" s="48" t="s">
+      <c r="E94" s="45" t="s">
         <v>211</v>
       </c>
-      <c r="F94" s="48" t="s">
+      <c r="F94" s="45" t="s">
         <v>267</v>
       </c>
-      <c r="G94" s="48" t="s">
+      <c r="G94" s="45" t="s">
         <v>349</v>
       </c>
-      <c r="H94" s="48" t="s">
+      <c r="H94" s="45" t="s">
         <v>374</v>
       </c>
       <c r="I94" s="20" t="s">
         <v>439</v>
       </c>
-      <c r="J94" s="48" t="s">
+      <c r="J94" s="45" t="s">
         <v>485</v>
       </c>
-      <c r="K94" s="47" t="s">
+      <c r="K94" s="44" t="s">
         <v>517</v>
       </c>
-      <c r="L94" s="48">
+      <c r="L94" s="45">
         <v>1</v>
       </c>
-      <c r="M94" s="48">
+      <c r="M94" s="45">
         <f>L94*5</f>
         <v>5</v>
       </c>
-      <c r="N94" s="48" t="s">
-        <v>439</v>
-      </c>
-      <c r="O94" s="49" t="s">
-        <v>576</v>
-      </c>
-      <c r="P94" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q94" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="R94" s="51" t="s">
+      <c r="N94" s="45" t="s">
+        <v>439</v>
+      </c>
+      <c r="O94" s="46" t="s">
+        <v>576</v>
+      </c>
+      <c r="P94" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q94" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="R94" s="48" t="s">
         <v>575</v>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
       <c r="J95" s="20" t="s">
         <v>490</v>
       </c>
-      <c r="K95" s="46" t="s">
+      <c r="K95" s="43" t="s">
         <v>558</v>
       </c>
       <c r="L95" s="20">
@@ -7623,7 +7623,7 @@
       <c r="N95" s="20">
         <v>100</v>
       </c>
-      <c r="O95" s="53" t="s">
+      <c r="O95" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P95" s="21">
@@ -7665,7 +7665,7 @@
       <c r="J96" s="14" t="s">
         <v>491</v>
       </c>
-      <c r="K96" s="45" t="s">
+      <c r="K96" s="42" t="s">
         <v>532</v>
       </c>
       <c r="L96" s="14">
@@ -7678,7 +7678,7 @@
       <c r="N96" s="14">
         <v>100</v>
       </c>
-      <c r="O96" s="53" t="s">
+      <c r="O96" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P96" s="15">
@@ -7720,7 +7720,7 @@
       <c r="J97" s="20" t="s">
         <v>492</v>
       </c>
-      <c r="K97" s="46" t="s">
+      <c r="K97" s="43" t="s">
         <v>559</v>
       </c>
       <c r="L97" s="20">
@@ -7733,7 +7733,7 @@
       <c r="N97" s="20">
         <v>100</v>
       </c>
-      <c r="O97" s="53" t="s">
+      <c r="O97" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P97" s="21">
@@ -7775,7 +7775,7 @@
       <c r="J98" s="14" t="s">
         <v>493</v>
       </c>
-      <c r="K98" s="45" t="s">
+      <c r="K98" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L98" s="14">
@@ -7788,7 +7788,7 @@
       <c r="N98" s="14">
         <v>15</v>
       </c>
-      <c r="O98" s="53" t="s">
+      <c r="O98" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P98" s="15">
@@ -7830,7 +7830,7 @@
       <c r="J99" s="20" t="s">
         <v>494</v>
       </c>
-      <c r="K99" s="45" t="s">
+      <c r="K99" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L99" s="20">
@@ -7843,7 +7843,7 @@
       <c r="N99" s="20">
         <v>6</v>
       </c>
-      <c r="O99" s="53" t="s">
+      <c r="O99" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P99" s="21">
@@ -7885,7 +7885,7 @@
       <c r="J100" s="14" t="s">
         <v>495</v>
       </c>
-      <c r="K100" s="45" t="s">
+      <c r="K100" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L100" s="14">
@@ -7898,7 +7898,7 @@
       <c r="N100" s="14">
         <v>10</v>
       </c>
-      <c r="O100" s="53" t="s">
+      <c r="O100" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P100" s="15">
@@ -7940,7 +7940,7 @@
       <c r="J101" s="20" t="s">
         <v>496</v>
       </c>
-      <c r="K101" s="45" t="s">
+      <c r="K101" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L101" s="20">
@@ -7953,7 +7953,7 @@
       <c r="N101" s="20">
         <v>6</v>
       </c>
-      <c r="O101" s="53" t="s">
+      <c r="O101" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P101" s="21">
@@ -7995,7 +7995,7 @@
       <c r="J102" s="14" t="s">
         <v>497</v>
       </c>
-      <c r="K102" s="45" t="s">
+      <c r="K102" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L102" s="14">
@@ -8008,7 +8008,7 @@
       <c r="N102" s="14">
         <v>6</v>
       </c>
-      <c r="O102" s="53" t="s">
+      <c r="O102" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P102" s="15">
@@ -8050,7 +8050,7 @@
       <c r="J103" s="20" t="s">
         <v>498</v>
       </c>
-      <c r="K103" s="45" t="s">
+      <c r="K103" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L103" s="20">
@@ -8063,7 +8063,7 @@
       <c r="N103" s="20">
         <v>6</v>
       </c>
-      <c r="O103" s="53" t="s">
+      <c r="O103" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P103" s="21">
@@ -8105,7 +8105,7 @@
       <c r="J104" s="14" t="s">
         <v>499</v>
       </c>
-      <c r="K104" s="45" t="s">
+      <c r="K104" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L104" s="14">
@@ -8118,7 +8118,7 @@
       <c r="N104" s="14">
         <v>6</v>
       </c>
-      <c r="O104" s="53" t="s">
+      <c r="O104" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P104" s="15">
@@ -8160,7 +8160,7 @@
       <c r="J105" s="20" t="s">
         <v>500</v>
       </c>
-      <c r="K105" s="45" t="s">
+      <c r="K105" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L105" s="20">
@@ -8173,7 +8173,7 @@
       <c r="N105" s="14">
         <v>11</v>
       </c>
-      <c r="O105" s="53" t="s">
+      <c r="O105" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P105" s="15">
@@ -8215,7 +8215,7 @@
       <c r="J106" s="14" t="s">
         <v>501</v>
       </c>
-      <c r="K106" s="45" t="s">
+      <c r="K106" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L106" s="14">
@@ -8228,7 +8228,7 @@
       <c r="N106" s="20">
         <v>6</v>
       </c>
-      <c r="O106" s="53" t="s">
+      <c r="O106" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P106" s="21">
@@ -8270,7 +8270,7 @@
       <c r="J107" s="14" t="s">
         <v>583</v>
       </c>
-      <c r="K107" s="45" t="s">
+      <c r="K107" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L107" s="20">
@@ -8283,7 +8283,7 @@
       <c r="N107" s="14">
         <v>6</v>
       </c>
-      <c r="O107" s="53" t="s">
+      <c r="O107" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P107" s="15">
@@ -8325,7 +8325,7 @@
       <c r="J108" s="14" t="s">
         <v>588</v>
       </c>
-      <c r="K108" s="45" t="s">
+      <c r="K108" s="42" t="s">
         <v>439</v>
       </c>
       <c r="L108" s="14">
@@ -8338,7 +8338,7 @@
       <c r="N108" s="14">
         <v>20</v>
       </c>
-      <c r="O108" s="53" t="s">
+      <c r="O108" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P108" s="15">
@@ -8359,50 +8359,50 @@
       <c r="C109" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="D109" s="48" t="s">
+      <c r="D109" s="45" t="s">
         <v>128</v>
       </c>
-      <c r="E109" s="48" t="s">
+      <c r="E109" s="45" t="s">
         <v>230</v>
       </c>
-      <c r="F109" s="48" t="s">
+      <c r="F109" s="45" t="s">
         <v>282</v>
       </c>
-      <c r="G109" s="48" t="s">
+      <c r="G109" s="45" t="s">
         <v>367</v>
       </c>
-      <c r="H109" s="48" t="s">
+      <c r="H109" s="45" t="s">
         <v>411</v>
       </c>
       <c r="I109" s="20" t="s">
         <v>439</v>
       </c>
-      <c r="J109" s="48" t="s">
+      <c r="J109" s="45" t="s">
         <v>502</v>
       </c>
-      <c r="K109" s="47" t="s">
+      <c r="K109" s="44" t="s">
         <v>517</v>
       </c>
-      <c r="L109" s="48">
+      <c r="L109" s="45">
         <v>1</v>
       </c>
-      <c r="M109" s="48">
+      <c r="M109" s="45">
         <f t="shared" ref="M109" si="100">L109*5</f>
         <v>5</v>
       </c>
-      <c r="N109" s="48" t="s">
-        <v>439</v>
-      </c>
-      <c r="O109" s="49" t="s">
-        <v>576</v>
-      </c>
-      <c r="P109" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q109" s="50" t="s">
-        <v>439</v>
-      </c>
-      <c r="R109" s="51" t="s">
+      <c r="N109" s="45" t="s">
+        <v>439</v>
+      </c>
+      <c r="O109" s="46" t="s">
+        <v>576</v>
+      </c>
+      <c r="P109" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q109" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="R109" s="48" t="s">
         <v>575</v>
       </c>
     </row>
@@ -8436,7 +8436,7 @@
       <c r="J110" s="14" t="s">
         <v>503</v>
       </c>
-      <c r="K110" s="45" t="s">
+      <c r="K110" s="42" t="s">
         <v>560</v>
       </c>
       <c r="L110" s="14">
@@ -8449,7 +8449,7 @@
       <c r="N110" s="20">
         <v>10</v>
       </c>
-      <c r="O110" s="53" t="s">
+      <c r="O110" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P110" s="21">
@@ -8491,7 +8491,7 @@
       <c r="J111" s="20" t="s">
         <v>504</v>
       </c>
-      <c r="K111" s="46" t="s">
+      <c r="K111" s="43" t="s">
         <v>561</v>
       </c>
       <c r="L111" s="20">
@@ -8504,7 +8504,7 @@
       <c r="N111" s="14">
         <v>10</v>
       </c>
-      <c r="O111" s="53" t="s">
+      <c r="O111" s="50" t="s">
         <v>576</v>
       </c>
       <c r="P111" s="15">
@@ -8530,14 +8530,14 @@
       <c r="K112" s="1"/>
       <c r="L112" s="1"/>
       <c r="M112" s="1"/>
-      <c r="N112" s="43" t="s">
+      <c r="N112" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="O112" s="44"/>
-      <c r="P112" s="44"/>
+      <c r="O112" s="53"/>
+      <c r="P112" s="53"/>
       <c r="Q112" s="18">
         <f>SUM(Q8:Q111)</f>
-        <v>376.17820000000006</v>
+        <v>381.32620000000003</v>
       </c>
       <c r="R112" s="1"/>
     </row>
@@ -8555,14 +8555,14 @@
       <c r="K113" s="1"/>
       <c r="L113" s="1"/>
       <c r="M113" s="1"/>
-      <c r="N113" s="43" t="s">
+      <c r="N113" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="O113" s="44"/>
-      <c r="P113" s="44"/>
+      <c r="O113" s="53"/>
+      <c r="P113" s="53"/>
       <c r="Q113" s="19">
         <f>Q112/5</f>
-        <v>75.235640000000018</v>
+        <v>76.265240000000006</v>
       </c>
       <c r="R113" s="1"/>
     </row>

</xml_diff>